<commit_message>
Add photos for all 69 employees in FINAL file
- Sourced every existing employee's photo from uploaded 'details (3)' file
  (parsed 61 in-cell richData images + 5 floating drawing images)
- New Momo Box staff (Gopal, Manas, Sunil) keep their PDF photos
- Embedded as standard floating images so they render in Excel & Google Sheets
- Compressed photos (~240px JPEG) -> file ~400KB
- Retained S.No fix, Aadhaar-only, brand banding, frozen header
</commit_message>
<xml_diff>
--- a/Azimuth Food Street Staff FRS details (FINAL).xlsx
+++ b/Azimuth Food Street Staff FRS details (FINAL).xlsx
@@ -360,17 +360,1242 @@
     <from>
       <col>5</col>
       <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="914400" cy="742950"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="714375" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>5</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="914400" cy="762000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>6</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="885825" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="914400" cy="828675"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="5" name="Image 5" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>8</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="914400" cy="752475"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="6" name="Image 6" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>9</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="371475" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="7" name="Image 7" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>10</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="914400" cy="733425"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="8" name="Image 8" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>11</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="914400" cy="809625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="9" name="Image 9" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId9"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>12</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="838200" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="10" name="Image 10" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId10"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>13</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="838200" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="11" name="Image 11" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId11"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>14</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="838200" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="12" name="Image 12" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId12"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>15</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="838200" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="13" name="Image 13" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId13"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>16</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="914400" cy="762000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="14" name="Image 14" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId14"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>17</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="838200" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="15" name="Image 15" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId15"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>18</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="838200" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="16" name="Image 16" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId16"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>19</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="838200" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="17" name="Image 17" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId17"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>20</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="838200" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="18" name="Image 18" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId18"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="838200" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="19" name="Image 19" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId19"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>22</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="838200" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="20" name="Image 20" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId20"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>23</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="904875" cy="762000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="21" name="Image 21" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId21"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>24</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="800100" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="22" name="Image 22" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId22"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="752475" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="23" name="Image 23" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId23"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>26</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="838200" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="24" name="Image 24" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId24"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>27</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="638175" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="25" name="Image 25" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId25"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>28</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="666750" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="26" name="Image 26" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId26"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>29</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="628650" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="27" name="Image 27" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId27"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>30</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="647700" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="28" name="Image 28" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId28"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>31</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="647700" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="29" name="Image 29" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId29"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>32</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="647700" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="30" name="Image 30" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId30"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>33</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="619125" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="31" name="Image 31" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId31"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>34</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="742950" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="32" name="Image 32" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId32"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>35</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="838200" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="33" name="Image 33" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId33"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>36</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="628650" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="34" name="Image 34" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId34"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>37</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="619125" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="35" name="Image 35" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId35"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>38</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="628650" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="36" name="Image 36" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId36"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>39</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="466725" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="37" name="Image 37" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId37"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>40</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="895350" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="38" name="Image 38" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId38"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>41</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="704850" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="39" name="Image 39" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId39"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>42</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="685800" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="40" name="Image 40" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId40"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>43</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="838200" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="41" name="Image 41" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId41"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>44</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="466725" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="42" name="Image 42" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId42"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>45</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="466725" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="43" name="Image 43" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId43"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>46</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="628650" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="44" name="Image 44" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId44"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>47</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="742950" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="45" name="Image 45" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId45"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>48</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="733425" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="46" name="Image 46" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId46"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>49</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="628650" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="47" name="Image 47" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId47"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>50</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="466725" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="48" name="Image 48" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId48"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>51</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="628650" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="49" name="Image 49" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId49"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
       <row>52</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="847725" cy="838200"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="1" name="Image 1" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
+        <cNvPr id="50" name="Image 50" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId50"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -391,11 +1616,11 @@
     <ext cx="704850" cy="838200"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="2" name="Image 2" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId2"/>
+        <cNvPr id="51" name="Image 51" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId51"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -416,11 +1641,11 @@
     <ext cx="685800" cy="838200"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="3" name="Image 3" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId3"/>
+        <cNvPr id="52" name="Image 52" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId52"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -441,11 +1666,11 @@
     <ext cx="466725" cy="838200"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="4" name="Image 4" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId4"/>
+        <cNvPr id="53" name="Image 53" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId53"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -466,11 +1691,11 @@
     <ext cx="666750" cy="838200"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="5" name="Image 5" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId5"/>
+        <cNvPr id="54" name="Image 54" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId54"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -491,11 +1716,11 @@
     <ext cx="628650" cy="838200"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="6" name="Image 6" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId6"/>
+        <cNvPr id="55" name="Image 55" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId55"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -516,11 +1741,11 @@
     <ext cx="628650" cy="838200"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="7" name="Image 7" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId7"/>
+        <cNvPr id="56" name="Image 56" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId56"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -541,11 +1766,311 @@
     <ext cx="628650" cy="838200"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="8" name="Image 8" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId8"/>
+        <cNvPr id="57" name="Image 57" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId57"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>60</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="628650" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="58" name="Image 58" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId58"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>61</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="476250" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="59" name="Image 59" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId59"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>62</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="714375" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="60" name="Image 60" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId60"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>63</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="61" name="Image 61" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId61"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>64</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="809625" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="62" name="Image 62" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId62"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>65</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="466725" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="63" name="Image 63" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId63"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>66</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="733425" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="64" name="Image 64" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId64"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>67</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="371475" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="65" name="Image 65" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId65"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>68</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="466725" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="66" name="Image 66" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId66"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>69</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="466725" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="67" name="Image 67" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId67"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>70</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="466725" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="68" name="Image 68" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId68"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>71</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="647700" cy="838200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="69" name="Image 69" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId69"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>

</xml_diff>